<commit_message>
compare108: report genes missing from the ORP count as masking by --top 0.1
The merge trace shows 78% of genes found among component hits but not ORP's
sit inside an ORP contig whose stronger hit to a related protein hides them;
at most 12% (median 77 per run) have no match in ORP. Section 4.3, the Table 2
caption, Methods and the polyploid paragraph now say so; S1 gains sheet
Gene_masking, built by explain_gene_masking.py.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiments/compare108/handoff/paper_20261023/ORP_4.0.0_lineage_results.xlsx
+++ b/experiments/compare108/handoff/paper_20261023/ORP_4.0.0_lineage_results.xlsx
@@ -16,8 +16,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ORP_vs_assembler" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ORP_vs_best_single" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Components" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings_dev30_vs_400" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RunTime" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gene_masking" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings_dev30_vs_400" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RunTime" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +44,9 @@
     <font>
       <name val="Arial"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -65,12 +69,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -436,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -540,48 +550,60 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Statistics</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Two-sided Wilcoxon signed-rank tests on paired values; Benjamini-Hochberg q within each Table 1 panel (11 metrics) or within each assembler (11 metrics).</t>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Gene_masking</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>For each Swiss-Prot gene among a component's DIAMOND hits (rerun with ORP's settings) but not ORP's, one component contig was located in the ORP assembly with blastn. Masked: matched at &gt;=95% identity over &gt;=90% of its length, with the gene's bitscore below 90% of the ORP contig's best (--top 0.1). No hit: the ORP contig has no hit. Unresolved: matched, gene within 10% but not reported. No match: no ORP match at that threshold (upper bound on sequence lost; one contig tested per gene). Built by explain_gene_masking.py from merge_trace (2026-10-23).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Values</t>
+          <t>Statistics</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>All cells are values computed in Python.</t>
+          <t>Two-sided Wilcoxon signed-rank tests on paired values; Benjamini-Hochberg q within each Table 1 panel (11 metrics) or within each assembler (11 metrics).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Sheets</t>
+          <t>Values</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Summary; Table1a; Table1b; Datasets; Groups; ORP_vs_assembler; ORP_vs_best_single; Components; Settings_dev30_vs_400 (first 50 datasets only); RunTime (per-step hours and CPU-hours for the first 50 only).</t>
+          <t>All cells are values computed in Python.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>Sheets</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Summary; Table1a; Table1b; Datasets; Groups; ORP_vs_assembler; ORP_vs_best_single; Components; Gene_masking (Section 4.3: genes among component hits but not ORP hits, by cause); Settings_dev30_vs_400 (first 50 datasets only); RunTime (per-step hours and CPU-hours for the first 50 only).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
           <t>Known caveats</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>tsa_GAGE reads are Apiospora malaysiana (ascomycete) but both assemblies were scored against agaricales_odb12.2. TSA assemblies are curated (no contigs &lt; 200 bp). tsa_GAQK excluded (R2 reads 62 bp).</t>
         </is>
@@ -593,6 +615,2444 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J60"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Organism</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Pair</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>SRA run</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Genes missing from ORP count</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Masked by --top 0.1</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>No hit on longer ORP contig</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Hit omitted, unresolved</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>No match in ORP (upper bound on sequence lost)</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Fraction with no match</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>echinodermata</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Apostichopus japonicus</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>tsa_GAVS</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>SRR1139215</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1378</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G2" t="n">
+        <v>44</v>
+      </c>
+      <c r="H2" t="n">
+        <v>122</v>
+      </c>
+      <c r="I2" t="n">
+        <v>112</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.081</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>echinodermata</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Asterias amurensis</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>tsa_GAVJ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>SRR1139201</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>963</v>
+      </c>
+      <c r="F3" t="n">
+        <v>778</v>
+      </c>
+      <c r="G3" t="n">
+        <v>40</v>
+      </c>
+      <c r="H3" t="n">
+        <v>69</v>
+      </c>
+      <c r="I3" t="n">
+        <v>76</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.079</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>echinodermata</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Eucidaris tribuloides</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>tsa_GAZP</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>SRR1138704</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>574</v>
+      </c>
+      <c r="F4" t="n">
+        <v>468</v>
+      </c>
+      <c r="G4" t="n">
+        <v>24</v>
+      </c>
+      <c r="H4" t="n">
+        <v>51</v>
+      </c>
+      <c r="I4" t="n">
+        <v>31</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.054</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>echinodermata</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Luidia clathrata</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>tsa_GAVQ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SRR1139195</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1018</v>
+      </c>
+      <c r="F5" t="n">
+        <v>773</v>
+      </c>
+      <c r="G5" t="n">
+        <v>58</v>
+      </c>
+      <c r="H5" t="n">
+        <v>109</v>
+      </c>
+      <c r="I5" t="n">
+        <v>78</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.077</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>echinodermata</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Lytechinus variegatus</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>tsa_GAUR</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>SRR1139214</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1058</v>
+      </c>
+      <c r="F6" t="n">
+        <v>881</v>
+      </c>
+      <c r="G6" t="n">
+        <v>43</v>
+      </c>
+      <c r="H6" t="n">
+        <v>69</v>
+      </c>
+      <c r="I6" t="n">
+        <v>65</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.061</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>echinodermata</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ophiocoma echinata</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>tsa_GAUQ</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>SRR1138707</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1091</v>
+      </c>
+      <c r="F7" t="n">
+        <v>875</v>
+      </c>
+      <c r="G7" t="n">
+        <v>47</v>
+      </c>
+      <c r="H7" t="n">
+        <v>75</v>
+      </c>
+      <c r="I7" t="n">
+        <v>94</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>echinodermata</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Oxycomanthus japonicus</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>tsa_GAZO</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>SRR1138706</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>845</v>
+      </c>
+      <c r="F8" t="n">
+        <v>726</v>
+      </c>
+      <c r="G8" t="n">
+        <v>19</v>
+      </c>
+      <c r="H8" t="n">
+        <v>74</v>
+      </c>
+      <c r="I8" t="n">
+        <v>26</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.031</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>echinodermata</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Patiria miniata</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>tsa_GAWB</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>SRR1138705</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1329</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1094</v>
+      </c>
+      <c r="G9" t="n">
+        <v>55</v>
+      </c>
+      <c r="H9" t="n">
+        <v>89</v>
+      </c>
+      <c r="I9" t="n">
+        <v>91</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.068</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>echinodermata</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Sclerodactyla briareus</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>tsa_GAUT</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>SRR1139189</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>735</v>
+      </c>
+      <c r="F10" t="n">
+        <v>596</v>
+      </c>
+      <c r="G10" t="n">
+        <v>37</v>
+      </c>
+      <c r="H10" t="n">
+        <v>67</v>
+      </c>
+      <c r="I10" t="n">
+        <v>35</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.048</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>echinodermata</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Sphaerechinus granularis</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>tsa_GAVR</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>SRR1139199</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1101</v>
+      </c>
+      <c r="F11" t="n">
+        <v>872</v>
+      </c>
+      <c r="G11" t="n">
+        <v>55</v>
+      </c>
+      <c r="H11" t="n">
+        <v>81</v>
+      </c>
+      <c r="I11" t="n">
+        <v>93</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.08400000000000001</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>embryophyta</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Aeginetia indica</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>orp_DRR082659</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>DRR082659</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>1255</v>
+      </c>
+      <c r="F12" t="n">
+        <v>910</v>
+      </c>
+      <c r="G12" t="n">
+        <v>51</v>
+      </c>
+      <c r="H12" t="n">
+        <v>85</v>
+      </c>
+      <c r="I12" t="n">
+        <v>209</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.167</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>embryophyta</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Arachis hypogaea</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>tsa_GAIG</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>SRR827601</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1067</v>
+      </c>
+      <c r="F13" t="n">
+        <v>867</v>
+      </c>
+      <c r="G13" t="n">
+        <v>28</v>
+      </c>
+      <c r="H13" t="n">
+        <v>111</v>
+      </c>
+      <c r="I13" t="n">
+        <v>61</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.057</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>embryophyta</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Avena sativa</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>tsa_GAJE</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>SRR850241</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>1340</v>
+      </c>
+      <c r="F14" t="n">
+        <v>936</v>
+      </c>
+      <c r="G14" t="n">
+        <v>55</v>
+      </c>
+      <c r="H14" t="n">
+        <v>82</v>
+      </c>
+      <c r="I14" t="n">
+        <v>267</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.199</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>embryophyta</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Brassica juncea</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>tsa_GBEP</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>SRR1265953</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>475</v>
+      </c>
+      <c r="F15" t="n">
+        <v>316</v>
+      </c>
+      <c r="G15" t="n">
+        <v>21</v>
+      </c>
+      <c r="H15" t="n">
+        <v>19</v>
+      </c>
+      <c r="I15" t="n">
+        <v>119</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.251</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>embryophyta</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Capsicum annuum</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>tsa_GAXU</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>SRR1123893</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>852</v>
+      </c>
+      <c r="F16" t="n">
+        <v>539</v>
+      </c>
+      <c r="G16" t="n">
+        <v>33</v>
+      </c>
+      <c r="H16" t="n">
+        <v>49</v>
+      </c>
+      <c r="I16" t="n">
+        <v>231</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.271</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>embryophyta</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Cephalotus follicularis</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>orp_DRR053698</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>DRR053698</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>1016</v>
+      </c>
+      <c r="F17" t="n">
+        <v>812</v>
+      </c>
+      <c r="G17" t="n">
+        <v>24</v>
+      </c>
+      <c r="H17" t="n">
+        <v>70</v>
+      </c>
+      <c r="I17" t="n">
+        <v>110</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.108</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>embryophyta</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Cocos nucifera</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>tsa_GABT</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>SRR606452</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>858</v>
+      </c>
+      <c r="F18" t="n">
+        <v>722</v>
+      </c>
+      <c r="G18" t="n">
+        <v>16</v>
+      </c>
+      <c r="H18" t="n">
+        <v>53</v>
+      </c>
+      <c r="I18" t="n">
+        <v>67</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.078</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>embryophyta</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Hevea brasiliensis</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>orp_DRR069093</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>DRR069093</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>1126</v>
+      </c>
+      <c r="F19" t="n">
+        <v>884</v>
+      </c>
+      <c r="G19" t="n">
+        <v>31</v>
+      </c>
+      <c r="H19" t="n">
+        <v>50</v>
+      </c>
+      <c r="I19" t="n">
+        <v>161</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.143</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>embryophyta</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Lotus corniculatus</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>tsa_GACB</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>SRR364671</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>739</v>
+      </c>
+      <c r="F20" t="n">
+        <v>600</v>
+      </c>
+      <c r="G20" t="n">
+        <v>33</v>
+      </c>
+      <c r="H20" t="n">
+        <v>73</v>
+      </c>
+      <c r="I20" t="n">
+        <v>33</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.045</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>embryophyta</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Musa ABB Group</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>tsa_GABH</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>SRR516083</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>1403</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1041</v>
+      </c>
+      <c r="G21" t="n">
+        <v>50</v>
+      </c>
+      <c r="H21" t="n">
+        <v>83</v>
+      </c>
+      <c r="I21" t="n">
+        <v>229</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.163</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>embryophyta</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Nicotiana tabacum</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>orp_SRR3499127</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>SRR3499127</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>1031</v>
+      </c>
+      <c r="F22" t="n">
+        <v>774</v>
+      </c>
+      <c r="G22" t="n">
+        <v>42</v>
+      </c>
+      <c r="H22" t="n">
+        <v>64</v>
+      </c>
+      <c r="I22" t="n">
+        <v>151</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.146</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>embryophyta</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Plukenetia volubilis</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>tsa_GADC</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>SRR627546</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>710</v>
+      </c>
+      <c r="F23" t="n">
+        <v>550</v>
+      </c>
+      <c r="G23" t="n">
+        <v>28</v>
+      </c>
+      <c r="H23" t="n">
+        <v>56</v>
+      </c>
+      <c r="I23" t="n">
+        <v>76</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.107</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>embryophyta</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Thlaspi arvense</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>tsa_GAKE</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>SRR802670</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>1074</v>
+      </c>
+      <c r="F24" t="n">
+        <v>793</v>
+      </c>
+      <c r="G24" t="n">
+        <v>18</v>
+      </c>
+      <c r="H24" t="n">
+        <v>55</v>
+      </c>
+      <c r="I24" t="n">
+        <v>208</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.194</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>embryophyta</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Vigna angularis</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>orp_DRR031870</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>DRR031870</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>798</v>
+      </c>
+      <c r="F25" t="n">
+        <v>572</v>
+      </c>
+      <c r="G25" t="n">
+        <v>31</v>
+      </c>
+      <c r="H25" t="n">
+        <v>48</v>
+      </c>
+      <c r="I25" t="n">
+        <v>147</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0.184</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>insecta</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Anopheles gambiae</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>orp_ERR489297</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>ERR489297</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>1136</v>
+      </c>
+      <c r="F26" t="n">
+        <v>963</v>
+      </c>
+      <c r="G26" t="n">
+        <v>32</v>
+      </c>
+      <c r="H26" t="n">
+        <v>53</v>
+      </c>
+      <c r="I26" t="n">
+        <v>88</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0.077</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>insecta</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Archaeopsylla erinacei</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>tsa_GABB</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>SRR578730</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>467</v>
+      </c>
+      <c r="F27" t="n">
+        <v>352</v>
+      </c>
+      <c r="G27" t="n">
+        <v>28</v>
+      </c>
+      <c r="H27" t="n">
+        <v>53</v>
+      </c>
+      <c r="I27" t="n">
+        <v>34</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0.073</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>insecta</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Bemisia tabaci</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>tsa_GAPQ</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>SRR835756</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>584</v>
+      </c>
+      <c r="F28" t="n">
+        <v>514</v>
+      </c>
+      <c r="G28" t="n">
+        <v>15</v>
+      </c>
+      <c r="H28" t="n">
+        <v>39</v>
+      </c>
+      <c r="I28" t="n">
+        <v>16</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0.027</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>insecta</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Chilo suppressalis</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>tsa_GAJS</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>SRR651040</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>707</v>
+      </c>
+      <c r="F29" t="n">
+        <v>587</v>
+      </c>
+      <c r="G29" t="n">
+        <v>32</v>
+      </c>
+      <c r="H29" t="n">
+        <v>61</v>
+      </c>
+      <c r="I29" t="n">
+        <v>27</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0.038</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>insecta</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Chrysopa pallens</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>tsa_GAGF</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>SRR653211</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>607</v>
+      </c>
+      <c r="F30" t="n">
+        <v>476</v>
+      </c>
+      <c r="G30" t="n">
+        <v>25</v>
+      </c>
+      <c r="H30" t="n">
+        <v>64</v>
+      </c>
+      <c r="I30" t="n">
+        <v>42</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0.06900000000000001</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>insecta</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Cotesia vestalis</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>tsa_GAKG</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>SRR770031</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>902</v>
+      </c>
+      <c r="F31" t="n">
+        <v>744</v>
+      </c>
+      <c r="G31" t="n">
+        <v>13</v>
+      </c>
+      <c r="H31" t="n">
+        <v>68</v>
+      </c>
+      <c r="I31" t="n">
+        <v>77</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>insecta</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Drosophila pseudoananassae nigrens</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>tsa_GADR</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>SRR544889</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>715</v>
+      </c>
+      <c r="F32" t="n">
+        <v>618</v>
+      </c>
+      <c r="G32" t="n">
+        <v>21</v>
+      </c>
+      <c r="H32" t="n">
+        <v>45</v>
+      </c>
+      <c r="I32" t="n">
+        <v>31</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0.043</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>insecta</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Kerria lacca</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>tsa_GBDO</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>SRR1104126</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>625</v>
+      </c>
+      <c r="F33" t="n">
+        <v>463</v>
+      </c>
+      <c r="G33" t="n">
+        <v>16</v>
+      </c>
+      <c r="H33" t="n">
+        <v>52</v>
+      </c>
+      <c r="I33" t="n">
+        <v>94</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>insecta</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Leptopilina heterotoma</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>tsa_GAJC</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>SRR559224</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>974</v>
+      </c>
+      <c r="F34" t="n">
+        <v>727</v>
+      </c>
+      <c r="G34" t="n">
+        <v>27</v>
+      </c>
+      <c r="H34" t="n">
+        <v>59</v>
+      </c>
+      <c r="I34" t="n">
+        <v>161</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0.165</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>insecta</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Sipyloidea sipylus</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>tsa_GAWF</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>SRR1172444</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>1053</v>
+      </c>
+      <c r="F35" t="n">
+        <v>891</v>
+      </c>
+      <c r="G35" t="n">
+        <v>25</v>
+      </c>
+      <c r="H35" t="n">
+        <v>58</v>
+      </c>
+      <c r="I35" t="n">
+        <v>79</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0.075</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>mammalia</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Callithrix jacchus</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>tsa_GAMP</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>SRR867044</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>212</v>
+      </c>
+      <c r="F36" t="n">
+        <v>166</v>
+      </c>
+      <c r="G36" t="n">
+        <v>8</v>
+      </c>
+      <c r="H36" t="n">
+        <v>23</v>
+      </c>
+      <c r="I36" t="n">
+        <v>15</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0.07099999999999999</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>mammalia</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Camelus bactrianus</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>tsa_GAFA</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>SRR527316</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>162</v>
+      </c>
+      <c r="F37" t="n">
+        <v>123</v>
+      </c>
+      <c r="G37" t="n">
+        <v>17</v>
+      </c>
+      <c r="H37" t="n">
+        <v>13</v>
+      </c>
+      <c r="I37" t="n">
+        <v>9</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0.056</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>mammalia</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Camelus dromedarius</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>tsa_GADW</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>SRR527279</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>170</v>
+      </c>
+      <c r="F38" t="n">
+        <v>135</v>
+      </c>
+      <c r="G38" t="n">
+        <v>6</v>
+      </c>
+      <c r="H38" t="n">
+        <v>14</v>
+      </c>
+      <c r="I38" t="n">
+        <v>15</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0.08799999999999999</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>mammalia</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Capra hircus</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>tsa_GAOE</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>SRR747797</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>241</v>
+      </c>
+      <c r="F39" t="n">
+        <v>175</v>
+      </c>
+      <c r="G39" t="n">
+        <v>9</v>
+      </c>
+      <c r="H39" t="n">
+        <v>23</v>
+      </c>
+      <c r="I39" t="n">
+        <v>34</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0.141</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>mammalia</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Mus musculus</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>orp_DRR036858</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>DRR036858</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>281</v>
+      </c>
+      <c r="F40" t="n">
+        <v>177</v>
+      </c>
+      <c r="G40" t="n">
+        <v>10</v>
+      </c>
+      <c r="H40" t="n">
+        <v>17</v>
+      </c>
+      <c r="I40" t="n">
+        <v>77</v>
+      </c>
+      <c r="J40" t="n">
+        <v>0.274</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>mammalia</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Mus musculus</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>orp_SRR2086412</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>SRR2086412</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>155</v>
+      </c>
+      <c r="F41" t="n">
+        <v>112</v>
+      </c>
+      <c r="G41" t="n">
+        <v>5</v>
+      </c>
+      <c r="H41" t="n">
+        <v>8</v>
+      </c>
+      <c r="I41" t="n">
+        <v>30</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0.194</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>mammalia</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Oryctolagus cuniculus</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>orp_SRR1789336</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>SRR1789336</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>223</v>
+      </c>
+      <c r="F42" t="n">
+        <v>172</v>
+      </c>
+      <c r="G42" t="n">
+        <v>21</v>
+      </c>
+      <c r="H42" t="n">
+        <v>14</v>
+      </c>
+      <c r="I42" t="n">
+        <v>16</v>
+      </c>
+      <c r="J42" t="n">
+        <v>0.07199999999999999</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>mammalia</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Pan troglodytes</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>tsa_GABC</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>SRR544868</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>207</v>
+      </c>
+      <c r="F43" t="n">
+        <v>171</v>
+      </c>
+      <c r="G43" t="n">
+        <v>6</v>
+      </c>
+      <c r="H43" t="n">
+        <v>19</v>
+      </c>
+      <c r="I43" t="n">
+        <v>11</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0.053</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Apiospora malaysiana</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>tsa_GAGE</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>SRR746797</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>402</v>
+      </c>
+      <c r="F44" t="n">
+        <v>347</v>
+      </c>
+      <c r="G44" t="n">
+        <v>12</v>
+      </c>
+      <c r="H44" t="n">
+        <v>21</v>
+      </c>
+      <c r="I44" t="n">
+        <v>22</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0.055</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Echinococcus multilocularis</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>orp_DRR030368</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>DRR030368</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>1475</v>
+      </c>
+      <c r="F45" t="n">
+        <v>1191</v>
+      </c>
+      <c r="G45" t="n">
+        <v>24</v>
+      </c>
+      <c r="H45" t="n">
+        <v>88</v>
+      </c>
+      <c r="I45" t="n">
+        <v>172</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0.117</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Echinogammarus veneris</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>tsa_GARO</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>SRR1050726</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>548</v>
+      </c>
+      <c r="F46" t="n">
+        <v>372</v>
+      </c>
+      <c r="G46" t="n">
+        <v>56</v>
+      </c>
+      <c r="H46" t="n">
+        <v>57</v>
+      </c>
+      <c r="I46" t="n">
+        <v>63</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0.115</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Entamoeba histolytica</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>orp_ERR058009</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>ERR058009</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>374</v>
+      </c>
+      <c r="F47" t="n">
+        <v>294</v>
+      </c>
+      <c r="G47" t="n">
+        <v>14</v>
+      </c>
+      <c r="H47" t="n">
+        <v>43</v>
+      </c>
+      <c r="I47" t="n">
+        <v>23</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0.061</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Heterorhabditis indica</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>orp_ERR1016675</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>ERR1016675</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>1240</v>
+      </c>
+      <c r="F48" t="n">
+        <v>823</v>
+      </c>
+      <c r="G48" t="n">
+        <v>44</v>
+      </c>
+      <c r="H48" t="n">
+        <v>70</v>
+      </c>
+      <c r="I48" t="n">
+        <v>303</v>
+      </c>
+      <c r="J48" t="n">
+        <v>0.244</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Phyllodoce medipapillata</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>orp_SRR2016923</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>SRR2016923</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>972</v>
+      </c>
+      <c r="F49" t="n">
+        <v>647</v>
+      </c>
+      <c r="G49" t="n">
+        <v>62</v>
+      </c>
+      <c r="H49" t="n">
+        <v>78</v>
+      </c>
+      <c r="I49" t="n">
+        <v>185</v>
+      </c>
+      <c r="J49" t="n">
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Schistosoma mansoni</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>orp_ERR1674585</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>ERR1674585</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>423</v>
+      </c>
+      <c r="F50" t="n">
+        <v>320</v>
+      </c>
+      <c r="G50" t="n">
+        <v>16</v>
+      </c>
+      <c r="H50" t="n">
+        <v>35</v>
+      </c>
+      <c r="I50" t="n">
+        <v>52</v>
+      </c>
+      <c r="J50" t="n">
+        <v>0.123</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Stegodyphus mimosarum</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>tsa_GAZR</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>SRR1015314</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>890</v>
+      </c>
+      <c r="F51" t="n">
+        <v>689</v>
+      </c>
+      <c r="G51" t="n">
+        <v>47</v>
+      </c>
+      <c r="H51" t="n">
+        <v>60</v>
+      </c>
+      <c r="I51" t="n">
+        <v>94</v>
+      </c>
+      <c r="J51" t="n">
+        <v>0.106</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>vertebrata</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Anolis carolinensis</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>tsa_GAGA</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>SRR389086</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>239</v>
+      </c>
+      <c r="F52" t="n">
+        <v>128</v>
+      </c>
+      <c r="G52" t="n">
+        <v>42</v>
+      </c>
+      <c r="H52" t="n">
+        <v>25</v>
+      </c>
+      <c r="I52" t="n">
+        <v>44</v>
+      </c>
+      <c r="J52" t="n">
+        <v>0.184</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>vertebrata</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Anolis carolinensis</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>tsa_GAGB</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>SRR389085</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>276</v>
+      </c>
+      <c r="F53" t="n">
+        <v>134</v>
+      </c>
+      <c r="G53" t="n">
+        <v>50</v>
+      </c>
+      <c r="H53" t="n">
+        <v>22</v>
+      </c>
+      <c r="I53" t="n">
+        <v>70</v>
+      </c>
+      <c r="J53" t="n">
+        <v>0.254</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>vertebrata</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Anoplopoma fimbria</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>tsa_GAJJ</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>SRR851004</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>577</v>
+      </c>
+      <c r="F54" t="n">
+        <v>424</v>
+      </c>
+      <c r="G54" t="n">
+        <v>16</v>
+      </c>
+      <c r="H54" t="n">
+        <v>57</v>
+      </c>
+      <c r="I54" t="n">
+        <v>80</v>
+      </c>
+      <c r="J54" t="n">
+        <v>0.139</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>vertebrata</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Latimeria chalumnae</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>tsa_GAAA</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>SRR401852</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>1821</v>
+      </c>
+      <c r="F55" t="n">
+        <v>1567</v>
+      </c>
+      <c r="G55" t="n">
+        <v>30</v>
+      </c>
+      <c r="H55" t="n">
+        <v>90</v>
+      </c>
+      <c r="I55" t="n">
+        <v>134</v>
+      </c>
+      <c r="J55" t="n">
+        <v>0.074</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>vertebrata</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Miichthys miiuy</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>tsa_GARA</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>SRR1060332</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>423</v>
+      </c>
+      <c r="F56" t="n">
+        <v>363</v>
+      </c>
+      <c r="G56" t="n">
+        <v>17</v>
+      </c>
+      <c r="H56" t="n">
+        <v>31</v>
+      </c>
+      <c r="I56" t="n">
+        <v>12</v>
+      </c>
+      <c r="J56" t="n">
+        <v>0.028</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>vertebrata</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Morone chrysops</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>tsa_GAZY</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>SRR1187194</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>932</v>
+      </c>
+      <c r="F57" t="n">
+        <v>717</v>
+      </c>
+      <c r="G57" t="n">
+        <v>20</v>
+      </c>
+      <c r="H57" t="n">
+        <v>45</v>
+      </c>
+      <c r="I57" t="n">
+        <v>150</v>
+      </c>
+      <c r="J57" t="n">
+        <v>0.161</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>vertebrata</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Morone saxatilis</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>tsa_GBAA</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>SRR1187193</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>948</v>
+      </c>
+      <c r="F58" t="n">
+        <v>719</v>
+      </c>
+      <c r="G58" t="n">
+        <v>23</v>
+      </c>
+      <c r="H58" t="n">
+        <v>63</v>
+      </c>
+      <c r="I58" t="n">
+        <v>143</v>
+      </c>
+      <c r="J58" t="n">
+        <v>0.151</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>vertebrata</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Oncorhynchus mykiss</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>orp_DRR046632</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>DRR046632</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>474</v>
+      </c>
+      <c r="F59" t="n">
+        <v>332</v>
+      </c>
+      <c r="G59" t="n">
+        <v>18</v>
+      </c>
+      <c r="H59" t="n">
+        <v>28</v>
+      </c>
+      <c r="I59" t="n">
+        <v>96</v>
+      </c>
+      <c r="J59" t="n">
+        <v>0.203</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>vertebrata</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Oreochromis niloticus</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>tsa_GAID</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>SRR797490</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>428</v>
+      </c>
+      <c r="F60" t="n">
+        <v>314</v>
+      </c>
+      <c r="G60" t="n">
+        <v>28</v>
+      </c>
+      <c r="H60" t="n">
+        <v>31</v>
+      </c>
+      <c r="I60" t="n">
+        <v>55</v>
+      </c>
+      <c r="J60" t="n">
+        <v>0.129</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6002,7 +8462,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>